<commit_message>
Aggiorna dashboard e dati · 2026-09-15 14:48:14
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -495,7 +495,7 @@
         <v>1000</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="G3">
         <f>MAX(0,E3-F3)</f>
@@ -3219,7 +3219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3309,6 +3309,42 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>c4172292-a096-4bb8-a330-2412f5a16bb3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n">
+        <v>46280.58472222222</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Colon keychain arancioni</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>145</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Porrtachiavi arancioni colon per notte dei ricercatori</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>c4172292-a096-4bb8-a330-2412f5a16bb3</t>
         </is>

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-15 15:15:34
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -604,13 +604,44 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>3ntr</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Giallo</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
       <c r="G6">
-        <f>IF(A6="","",MAX(0,E6-F6))</f>
+        <f>MAX(0,E6-F6)</f>
         <v/>
       </c>
       <c r="H6" s="5">
-        <f>IF(A6="","",IFERROR(G6/E6,0))</f>
-        <v/>
+        <f>IFERROR(G6/E6,0)</f>
+        <v/>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-15 15:26:03
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -645,16 +645,44 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>3ntr</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1000</v>
+      </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7">
-        <f>IF(A7="","",MAX(0,E7-F7))</f>
+        <f>MAX(0,E7-F7)</f>
         <v/>
       </c>
       <c r="H7" s="5">
-        <f>IF(A7="","",IFERROR(G7/E7,0))</f>
-        <v/>
+        <f>IFERROR(G7/E7,0)</f>
+        <v/>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-15 16:00:47
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -686,16 +686,44 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3ntr</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>fuchsia</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1000</v>
+      </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8">
-        <f>IF(A8="","",MAX(0,E8-F8))</f>
+        <f>MAX(0,E8-F8)</f>
         <v/>
       </c>
       <c r="H8" s="5">
-        <f>IF(A8="","",IFERROR(G8/E8,0))</f>
-        <v/>
+        <f>IFERROR(G8/E8,0)</f>
+        <v/>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-15 16:01:02
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -363,7 +363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J201"/>
+  <dimension ref="A1:K201"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -423,6 +423,11 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Archivio</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -723,6 +728,11 @@
       <c r="I8" t="inlineStr">
         <is>
           <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Eliminata</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-15 16:09:59
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -737,16 +737,44 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>3ntr</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Rosso</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1000</v>
+      </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9">
-        <f>IF(A9="","",MAX(0,E9-F9))</f>
+        <f>MAX(0,E9-F9)</f>
         <v/>
       </c>
       <c r="H9" s="5">
-        <f>IF(A9="","",IFERROR(G9/E9,0))</f>
-        <v/>
+        <f>IFERROR(G9/E9,0)</f>
+        <v/>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-15 16:22:09
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -778,16 +778,44 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>B009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3ntr</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Rosa</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1000</v>
+      </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10">
-        <f>IF(A10="","",MAX(0,E10-F10))</f>
+        <f>MAX(0,E10-F10)</f>
         <v/>
       </c>
       <c r="H10" s="5">
-        <f>IF(A10="","",IFERROR(G10/E10,0))</f>
-        <v/>
+        <f>IFERROR(G10/E10,0)</f>
+        <v/>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-15 16:25:51
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -819,16 +819,44 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>B010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3ntr</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Naturale</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1000</v>
+      </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11">
-        <f>IF(A11="","",MAX(0,E11-F11))</f>
+        <f>MAX(0,E11-F11)</f>
         <v/>
       </c>
       <c r="H11" s="5">
-        <f>IF(A11="","",IFERROR(G11/E11,0))</f>
-        <v/>
+        <f>IFERROR(G11/E11,0)</f>
+        <v/>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-16 10:14:59
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -454,7 +454,7 @@
         <v>5000</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="G2">
         <f>MAX(0,E2-F2)</f>
@@ -500,7 +500,7 @@
         <v>1000</v>
       </c>
       <c r="F3" t="n">
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="G3">
         <f>MAX(0,E3-F3)</f>
@@ -546,7 +546,7 @@
         <v>1000</v>
       </c>
       <c r="F4" t="n">
-        <v>219</v>
+        <v>319</v>
       </c>
       <c r="G4">
         <f>MAX(0,E4-F4)</f>
@@ -3400,7 +3400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3482,7 +3482,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>219</v>
+        <v>30</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -3518,7 +3518,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>145</v>
+        <v>50</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -3528,6 +3528,99 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>c4172292-a096-4bb8-a330-2412f5a16bb3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>46281.42638888889</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Scatole da D1 a D5 con inserti separati</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>36</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0a9569eb-86c6-44e5-b208-a297dfd89bf6</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="n">
+        <v>46281.42638888889</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Scatole da D1 a D5 con inserti separati</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>125</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0a9569eb-86c6-44e5-b208-a297dfd89bf6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n">
+        <v>46281.42638888889</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Scatole da D1 a D5 con inserti separati</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>289</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0a9569eb-86c6-44e5-b208-a297dfd89bf6</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-17 10:22:53
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Ugelli" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Stampe" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Liste" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pianificazione" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -3793,4 +3794,196 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID Pianificazione</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nome stampa</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Durata (min)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Inizio previsto</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ugello</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ID Bobina</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Materiale</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Grammi previsti</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Creata il</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>71d31883-77ba-4398-9dc9-8b313ee67220</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ScatoleP1P5_inserti</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1860</v>
+      </c>
+      <c r="D2" s="8" t="n">
+        <v>46282.4375</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Scatole palpable da P1 a P5</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="n">
+        <v>46282.43228212963</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>71d31883-77ba-4398-9dc9-8b313ee67220</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ScatoleP1P5_inserti</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1860</v>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>46282.4375</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Scatole palpable da P1 a P5</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="n">
+        <v>46282.43228212963</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>71d31883-77ba-4398-9dc9-8b313ee67220</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ScatoleP1P5_inserti</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1860</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>46282.4375</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Scatole palpable da P1 a P5</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="n">
+        <v>46282.43228212963</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-17 10:24:57
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -3802,7 +3802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3872,7 +3872,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46282.4375</v>
+        <v>46284.4375</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -3914,7 +3914,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46282.4375</v>
+        <v>46284.4375</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -3956,7 +3956,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46282.4375</v>
+        <v>46284.4375</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -3981,6 +3981,132 @@
       </c>
       <c r="J4" s="8" t="n">
         <v>46282.43228212963</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>58e8ef87-b799-4b9e-ac2d-62b2f4e2a9e5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ScatoleDAPAV1V2V3+inserti.3mf</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>46282.4375</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Scatole palpable DA PA V1 V2 V3</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>46282.43368086805</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>58e8ef87-b799-4b9e-ac2d-62b2f4e2a9e5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ScatoleDAPAV1V2V3+inserti.3mf</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>46282.4375</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Scatole palpable DA PA V1 V2 V3</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>46282.43368086805</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>58e8ef87-b799-4b9e-ac2d-62b2f4e2a9e5</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ScatoleDAPAV1V2V3+inserti.3mf</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>46282.4375</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Scatole palpable DA PA V1 V2 V3</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>46282.43368086805</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-17 10:46:59
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -3802,7 +3802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3872,7 +3872,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46284.4375</v>
+        <v>46284.73958333334</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -3914,7 +3914,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46284.4375</v>
+        <v>46284.73958333334</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -3956,7 +3956,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46284.4375</v>
+        <v>46284.73958333334</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -3998,7 +3998,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46282.4375</v>
+        <v>46283.40625</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4040,7 +4040,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46282.4375</v>
+        <v>46283.40625</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4082,7 +4082,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46282.4375</v>
+        <v>46283.40625</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
@@ -4107,6 +4107,141 @@
       </c>
       <c r="J7" s="8" t="n">
         <v>46282.43368086805</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="J8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="J9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="J10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>e690e833-17ba-4313-bf1d-5da3ed6efbba</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ScatoleD1D5_inserti</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1860</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>46281.43055555555</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>36</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Scatole palpable da D1 a D5 con inserti</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>46282.44827337963</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>e690e833-17ba-4313-bf1d-5da3ed6efbba</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ScatoleD1D5_inserti</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1860</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>46281.43055555555</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>125</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Scatole palpable da D1 a D5 con inserti</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>46282.44827337963</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>e690e833-17ba-4313-bf1d-5da3ed6efbba</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ScatoleD1D5_inserti</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1860</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>46281.43055555555</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>289</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Scatole palpable da D1 a D5 con inserti</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>46282.44827337963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-17 11:54:58
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -3802,7 +3802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4268,235 +4268,37 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>aa86423f-d4f6-4ecd-bc07-05219a350014</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>TEST</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>1200</v>
-      </c>
       <c r="D14" s="8" t="n"/>
-      <c r="E14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>10</v>
-      </c>
-      <c r="J14" s="8" t="n">
-        <v>46282.45661180556</v>
-      </c>
+      <c r="J14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>aa86423f-d4f6-4ecd-bc07-05219a350014</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>TEST</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>1200</v>
-      </c>
       <c r="D15" s="8" t="n"/>
-      <c r="E15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Supporto</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>20</v>
-      </c>
-      <c r="J15" s="8" t="n">
-        <v>46282.45661180556</v>
-      </c>
+      <c r="J15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>aa86423f-d4f6-4ecd-bc07-05219a350014</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>TEST</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>1200</v>
-      </c>
       <c r="D16" s="8" t="n"/>
-      <c r="E16" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>B003</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>10</v>
-      </c>
-      <c r="J16" s="8" t="n">
-        <v>46282.45661180556</v>
-      </c>
+      <c r="J16" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>89bcbc72-4a97-4033-8fb7-00c39e14637c</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>TEST</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>1260</v>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>46282.74305555555</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>10</v>
-      </c>
-      <c r="J17" s="8" t="n">
-        <v>46282.46811686343</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>SUBITO</t>
-        </is>
-      </c>
+      <c r="D17" s="8" t="n"/>
+      <c r="J17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>89bcbc72-4a97-4033-8fb7-00c39e14637c</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>TEST</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>1260</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>46282.74305555555</v>
-      </c>
-      <c r="E18" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Supporto</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>10</v>
-      </c>
-      <c r="J18" s="8" t="n">
-        <v>46282.46811686343</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>SUBITO</t>
-        </is>
-      </c>
+      <c r="D18" s="8" t="n"/>
+      <c r="J18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>89bcbc72-4a97-4033-8fb7-00c39e14637c</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>TEST</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>1260</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>46282.74305555555</v>
-      </c>
-      <c r="E19" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>B003</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>10</v>
-      </c>
-      <c r="J19" s="8" t="n">
-        <v>46282.46811686343</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>SUBITO</t>
-        </is>
-      </c>
+      <c r="D19" s="8" t="n"/>
+      <c r="J19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="J20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="J21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="J22" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-17 12:14:57
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -3802,7 +3802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3876,7 +3876,9 @@
       <c r="C2" t="n">
         <v>1860</v>
       </c>
-      <c r="D2" s="8" t="n"/>
+      <c r="D2" s="8" t="n">
+        <v>46282.72916666666</v>
+      </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
@@ -3921,7 +3923,9 @@
       <c r="C3" t="n">
         <v>1860</v>
       </c>
-      <c r="D3" s="8" t="n"/>
+      <c r="D3" s="8" t="n">
+        <v>46282.72916666666</v>
+      </c>
       <c r="E3" t="n">
         <v>2</v>
       </c>
@@ -3966,7 +3970,9 @@
       <c r="C4" t="n">
         <v>1860</v>
       </c>
-      <c r="D4" s="8" t="n"/>
+      <c r="D4" s="8" t="n">
+        <v>46282.72916666666</v>
+      </c>
       <c r="E4" t="n">
         <v>3</v>
       </c>
@@ -4038,7 +4044,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Urgente</t>
+          <t>SUBITO</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4089,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Urgente</t>
+          <t>SUBITO</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4134,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Urgente</t>
+          <t>SUBITO</t>
         </is>
       </c>
     </row>
@@ -4153,7 +4159,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1860</v>
+        <v>1815</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>46281.43055555555</v>
@@ -4195,7 +4201,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1860</v>
+        <v>1815</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>46281.43055555555</v>
@@ -4237,7 +4243,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1860</v>
+        <v>1815</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>46281.43055555555</v>
@@ -4299,6 +4305,411 @@
     </row>
     <row r="22">
       <c r="J22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>781cadba-d555-4a79-897d-1361ebfaeb0b</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Scatole GA + inserti + triangoli</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>10</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Scatola per palpable con GA e triangoli</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>46282.49938152778</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>SUBITO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>781cadba-d555-4a79-897d-1361ebfaeb0b</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Scatole GA + inserti + triangoli</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>10</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Scatola per palpable con GA e triangoli</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="n">
+        <v>46282.49938152778</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>SUBITO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>781cadba-d555-4a79-897d-1361ebfaeb0b</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Scatole GA + inserti + triangoli</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>10</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Scatola per palpable con GA e triangoli</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="n">
+        <v>46282.49938152778</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>SUBITO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>52447791-486f-45c5-a9f3-0d81985c5ecd</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Colon keychain 32arancioni e 32verdi</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1680</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>10</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Portachiavi colon per notte dei ricercatori</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="n">
+        <v>46282.49996001158</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>52447791-486f-45c5-a9f3-0d81985c5ecd</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Colon keychain 32arancioni e 32verdi</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1680</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>10</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Portachiavi colon per notte dei ricercatori</t>
+        </is>
+      </c>
+      <c r="J27" s="8" t="n">
+        <v>46282.49996001158</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>52447791-486f-45c5-a9f3-0d81985c5ecd</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Colon keychain 32arancioni e 32verdi</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1680</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>10</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Portachiavi colon per notte dei ricercatori</t>
+        </is>
+      </c>
+      <c r="J28" s="8" t="n">
+        <v>46282.49996001158</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>547a8bc6-095c-45b5-b678-e3f9bc5105a0</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Phantom_part3</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>4080</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>46284.13541666666</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>10</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>1 parte superiore phantom</t>
+        </is>
+      </c>
+      <c r="J29" s="8" t="n">
+        <v>46282.51013813657</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>547a8bc6-095c-45b5-b678-e3f9bc5105a0</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Phantom_part3</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>4080</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>46284.13541666666</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>10</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>1 parte superiore phantom</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="n">
+        <v>46282.51013813657</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>547a8bc6-095c-45b5-b678-e3f9bc5105a0</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Phantom_part3</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4080</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>46284.13541666666</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>10</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>1 parte superiore phantom</t>
+        </is>
+      </c>
+      <c r="J31" s="8" t="n">
+        <v>46282.51013813657</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-18 10:44:42
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -455,7 +455,7 @@
         <v>5000</v>
       </c>
       <c r="F2" t="n">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="G2">
         <f>MAX(0,E2-F2)</f>
@@ -501,7 +501,7 @@
         <v>1000</v>
       </c>
       <c r="F3" t="n">
-        <v>175</v>
+        <v>400</v>
       </c>
       <c r="G3">
         <f>MAX(0,E3-F3)</f>
@@ -547,7 +547,7 @@
         <v>1000</v>
       </c>
       <c r="F4" t="n">
-        <v>319</v>
+        <v>672</v>
       </c>
       <c r="G4">
         <f>MAX(0,E4-F4)</f>
@@ -675,7 +675,7 @@
         <v>1000</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="G7">
         <f>MAX(0,E7-F7)</f>
@@ -3401,7 +3401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3453,6 +3453,16 @@
           <t>ID Stampa</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Durata (min)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Inizio nel calendario</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="n"/>
@@ -3623,6 +3633,249 @@
         <is>
           <t>0a9569eb-86c6-44e5-b208-a297dfd89bf6</t>
         </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n">
+        <v>46281.4375</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ScatoleD1D5_inserti</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>36</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Scatole palpable da D1 a D5 con inserti</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>4b41cce9-5f53-4d19-9e69-0e8254ff52e7</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>1815</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>46281.4375</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ScatoleD1D5_inserti</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>125</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Scatole palpable da D1 a D5 con inserti</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>4b41cce9-5f53-4d19-9e69-0e8254ff52e7</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>1815</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
+        <v>46281.4375</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ScatoleD1D5_inserti</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>289</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Scatole palpable da D1 a D5 con inserti</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>4b41cce9-5f53-4d19-9e69-0e8254ff52e7</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>1815</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>46283.44583333333</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Colon keychain 32arancioni e 32verdi</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>B006</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>64</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Portachiavi colon per notte dei ricercatori</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ef366810-7fa1-4bd4-9bf9-8e3415150458</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>720</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>46282.72916666666</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n">
+        <v>46283.44583333333</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Colon keychain 32arancioni e 32verdi</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>100</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Portachiavi colon per notte dei ricercatori</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>ef366810-7fa1-4bd4-9bf9-8e3415150458</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>720</v>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>46282.72916666666</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>46283.44583333333</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Colon keychain 32arancioni e 32verdi</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>64</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Portachiavi colon per notte dei ricercatori</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ef366810-7fa1-4bd4-9bf9-8e3415150458</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>720</v>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>46282.72916666666</v>
       </c>
     </row>
   </sheetData>
@@ -3877,7 +4130,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46282.72916666666</v>
+        <v>46286.33333333334</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -3924,7 +4177,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46282.72916666666</v>
+        <v>46286.33333333334</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -3971,7 +4224,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46282.72916666666</v>
+        <v>46286.33333333334</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -4017,7 +4270,9 @@
       <c r="C5" t="n">
         <v>1800</v>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="8" t="n">
+        <v>46289.09375</v>
+      </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
@@ -4062,7 +4317,9 @@
       <c r="C6" t="n">
         <v>1800</v>
       </c>
-      <c r="D6" s="8" t="n"/>
+      <c r="D6" s="8" t="n">
+        <v>46289.09375</v>
+      </c>
       <c r="E6" t="n">
         <v>2</v>
       </c>
@@ -4107,7 +4364,9 @@
       <c r="C7" t="n">
         <v>1800</v>
       </c>
-      <c r="D7" s="8" t="n"/>
+      <c r="D7" s="8" t="n">
+        <v>46289.09375</v>
+      </c>
       <c r="E7" t="n">
         <v>3</v>
       </c>
@@ -4148,130 +4407,16 @@
       <c r="J10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>e690e833-17ba-4313-bf1d-5da3ed6efbba</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>ScatoleD1D5_inserti</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>1815</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>46281.43055555555</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>36</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Scatole palpable da D1 a D5 con inserti</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="n">
-        <v>46282.44827337963</v>
-      </c>
+      <c r="D11" s="8" t="n"/>
+      <c r="J11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>e690e833-17ba-4313-bf1d-5da3ed6efbba</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>ScatoleD1D5_inserti</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>1815</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>46281.43055555555</v>
-      </c>
-      <c r="E12" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Supporto</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>125</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Scatole palpable da D1 a D5 con inserti</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>46282.44827337963</v>
-      </c>
+      <c r="D12" s="8" t="n"/>
+      <c r="J12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>e690e833-17ba-4313-bf1d-5da3ed6efbba</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>ScatoleD1D5_inserti</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>1815</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>46281.43055555555</v>
-      </c>
-      <c r="E13" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>B003</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>289</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Scatole palpable da D1 a D5 con inserti</t>
-        </is>
-      </c>
-      <c r="J13" s="8" t="n">
-        <v>46282.44827337963</v>
-      </c>
+      <c r="D13" s="8" t="n"/>
+      <c r="J13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="D14" s="8" t="n"/>
@@ -4320,6 +4465,9 @@
       <c r="C23" t="n">
         <v>1800</v>
       </c>
+      <c r="D23" s="8" t="n">
+        <v>46287.64583333334</v>
+      </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
@@ -4364,6 +4512,9 @@
       <c r="C24" t="n">
         <v>1800</v>
       </c>
+      <c r="D24" s="8" t="n">
+        <v>46287.64583333334</v>
+      </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
@@ -4408,6 +4559,9 @@
       <c r="C25" t="n">
         <v>1800</v>
       </c>
+      <c r="D25" s="8" t="n">
+        <v>46287.64583333334</v>
+      </c>
       <c r="E25" t="n">
         <v>3</v>
       </c>
@@ -4439,136 +4593,16 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>52447791-486f-45c5-a9f3-0d81985c5ecd</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Colon keychain 32arancioni e 32verdi</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>1680</v>
-      </c>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H26" t="n">
-        <v>10</v>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Portachiavi colon per notte dei ricercatori</t>
-        </is>
-      </c>
-      <c r="J26" s="8" t="n">
-        <v>46282.49996001158</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Urgente</t>
-        </is>
-      </c>
+      <c r="D26" s="8" t="n"/>
+      <c r="J26" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>52447791-486f-45c5-a9f3-0d81985c5ecd</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Colon keychain 32arancioni e 32verdi</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>1680</v>
-      </c>
-      <c r="E27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Supporto</t>
-        </is>
-      </c>
-      <c r="H27" t="n">
-        <v>10</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Portachiavi colon per notte dei ricercatori</t>
-        </is>
-      </c>
-      <c r="J27" s="8" t="n">
-        <v>46282.49996001158</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Urgente</t>
-        </is>
-      </c>
+      <c r="D27" s="8" t="n"/>
+      <c r="J27" s="8" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>52447791-486f-45c5-a9f3-0d81985c5ecd</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Colon keychain 32arancioni e 32verdi</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>1680</v>
-      </c>
-      <c r="E28" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>B003</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H28" t="n">
-        <v>10</v>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Portachiavi colon per notte dei ricercatori</t>
-        </is>
-      </c>
-      <c r="J28" s="8" t="n">
-        <v>46282.49996001158</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Urgente</t>
-        </is>
-      </c>
+      <c r="D28" s="8" t="n"/>
+      <c r="J28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4585,7 +4619,7 @@
         <v>4080</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>46284.13541666666</v>
+        <v>46283.27083333334</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
@@ -4632,7 +4666,7 @@
         <v>4080</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>46284.13541666666</v>
+        <v>46283.27083333334</v>
       </c>
       <c r="E30" t="n">
         <v>2</v>
@@ -4679,7 +4713,7 @@
         <v>4080</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>46284.13541666666</v>
+        <v>46283.27083333334</v>
       </c>
       <c r="E31" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-18 10:47:06
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -818,6 +818,11 @@
           <t>Disponibile</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Eliminata</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -857,6 +862,11 @@
       <c r="I11" t="inlineStr">
         <is>
           <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Eliminata</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aggiorna dashboard e dati · 2026-09-18 10:58:19
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46286.33333333334</v>
+        <v>46286.27083333334</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46286.33333333334</v>
+        <v>46286.27083333334</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46286.33333333334</v>
+        <v>46286.27083333334</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:43:55
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46289.09375</v>
+        <v>46290.01041666666</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46289.09375</v>
+        <v>46290.01041666666</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46289.09375</v>
+        <v>46290.01041666666</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:44:16
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4065,7 +4065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4755,6 +4755,126 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>363c5463-4dda-4b36-a1a0-607308debf39</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TEST eliminare</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>180</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>10</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" s="8" t="n">
+        <v>46283.40574330497</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>SUBITO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>363c5463-4dda-4b36-a1a0-607308debf39</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TEST eliminare</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>180</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>10</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" s="8" t="n">
+        <v>46283.40574330497</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>SUBITO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>363c5463-4dda-4b36-a1a0-607308debf39</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>TEST eliminare</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>180</v>
+      </c>
+      <c r="E34" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>10</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" s="8" t="n">
+        <v>46283.40574330497</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>SUBITO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:44:24
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46287.64583333334</v>
+        <v>46288.57291666666</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46287.64583333334</v>
+        <v>46288.57291666666</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46287.64583333334</v>
+        <v>46288.57291666666</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>
@@ -4785,9 +4785,8 @@
       <c r="H32" t="n">
         <v>10</v>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" s="8" t="n">
-        <v>46283.40574330497</v>
+        <v>46283.40574331018</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -4825,9 +4824,8 @@
       <c r="H33" t="n">
         <v>10</v>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" s="8" t="n">
-        <v>46283.40574330497</v>
+        <v>46283.40574331018</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -4865,9 +4863,8 @@
       <c r="H34" t="n">
         <v>10</v>
       </c>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" s="8" t="n">
-        <v>46283.40574330497</v>
+        <v>46283.40574331018</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:44:28
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46286.27083333334</v>
+        <v>46287.20833333334</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46286.27083333334</v>
+        <v>46287.20833333334</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46286.27083333334</v>
+        <v>46287.20833333334</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:44:54
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4769,6 +4769,9 @@
       <c r="C32" t="n">
         <v>180</v>
       </c>
+      <c r="D32" s="8" t="n">
+        <v>46286.125</v>
+      </c>
       <c r="E32" t="n">
         <v>1</v>
       </c>
@@ -4808,6 +4811,9 @@
       <c r="C33" t="n">
         <v>180</v>
       </c>
+      <c r="D33" s="8" t="n">
+        <v>46286.125</v>
+      </c>
       <c r="E33" t="n">
         <v>2</v>
       </c>
@@ -4846,6 +4852,9 @@
       </c>
       <c r="C34" t="n">
         <v>180</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>46286.125</v>
       </c>
       <c r="E34" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:46:18
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46287.20833333334</v>
+        <v>46287.19791666666</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46287.20833333334</v>
+        <v>46287.19791666666</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46287.20833333334</v>
+        <v>46287.19791666666</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:56:27
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46287.19791666666</v>
+        <v>46286.28125</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46287.19791666666</v>
+        <v>46286.28125</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46287.19791666666</v>
+        <v>46286.28125</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:56:32
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46288.57291666666</v>
+        <v>46287.59375</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46288.57291666666</v>
+        <v>46287.59375</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46288.57291666666</v>
+        <v>46287.59375</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:56:40
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46287.59375</v>
+        <v>46287.67708333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46287.59375</v>
+        <v>46287.67708333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46287.59375</v>
+        <v>46287.67708333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:56:46
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46287.67708333334</v>
+        <v>46287.79166666666</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46287.67708333334</v>
+        <v>46287.79166666666</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46287.67708333334</v>
+        <v>46287.79166666666</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 09:56:52
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46290.01041666666</v>
+        <v>46289.36458333334</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46290.01041666666</v>
+        <v>46289.36458333334</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46290.01041666666</v>
+        <v>46289.36458333334</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:01:29
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46289.36458333334</v>
+        <v>46289.23958333334</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46289.36458333334</v>
+        <v>46289.23958333334</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46289.36458333334</v>
+        <v>46289.23958333334</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:01:30
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46289.23958333334</v>
+        <v>46289.13541666666</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46289.23958333334</v>
+        <v>46289.13541666666</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46289.23958333334</v>
+        <v>46289.13541666666</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:01:36
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46289.13541666666</v>
+        <v>46291.11458333334</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46289.13541666666</v>
+        <v>46291.11458333334</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46289.13541666666</v>
+        <v>46291.11458333334</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:01:43
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46291.11458333334</v>
+        <v>46290.0625</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46291.11458333334</v>
+        <v>46290.0625</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46291.11458333334</v>
+        <v>46290.0625</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:01:47
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46290.0625</v>
+        <v>46290.27083333334</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46290.0625</v>
+        <v>46290.27083333334</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46290.0625</v>
+        <v>46290.27083333334</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:02:04
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46290.27083333334</v>
+        <v>46289.23958333334</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46290.27083333334</v>
+        <v>46289.23958333334</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46290.27083333334</v>
+        <v>46289.23958333334</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:02:15
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46289.23958333334</v>
+        <v>46289.15625</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46289.23958333334</v>
+        <v>46289.15625</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46289.23958333334</v>
+        <v>46289.15625</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:02:33
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46287.79166666666</v>
+        <v>46287.58333333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46287.79166666666</v>
+        <v>46287.58333333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46287.79166666666</v>
+        <v>46287.58333333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:02:39
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46287.58333333334</v>
+        <v>46287.59375</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46287.58333333334</v>
+        <v>46287.59375</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46287.58333333334</v>
+        <v>46287.59375</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:02:46
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46287.59375</v>
+        <v>46287.64583333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46287.59375</v>
+        <v>46287.64583333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46287.59375</v>
+        <v>46287.64583333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:02:51
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46287.64583333334</v>
+        <v>46287.625</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46287.64583333334</v>
+        <v>46287.625</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46287.64583333334</v>
+        <v>46287.625</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:12:05
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46287.625</v>
+        <v>46287.67708333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46287.625</v>
+        <v>46287.67708333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46287.625</v>
+        <v>46287.67708333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:12:12
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46287.67708333334</v>
+        <v>46290.61458333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46287.67708333334</v>
+        <v>46290.61458333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46287.67708333334</v>
+        <v>46290.61458333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:12:15
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46289.15625</v>
+        <v>46288.16666666666</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46289.15625</v>
+        <v>46288.16666666666</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46289.15625</v>
+        <v>46288.16666666666</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:12:16
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46290.61458333334</v>
+        <v>46289.63541666666</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46290.61458333334</v>
+        <v>46289.63541666666</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46290.61458333334</v>
+        <v>46289.63541666666</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:12:21
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46289.63541666666</v>
+        <v>46289.44791666666</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46289.63541666666</v>
+        <v>46289.44791666666</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46289.63541666666</v>
+        <v>46289.44791666666</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:13:04
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46289.44791666666</v>
+        <v>46289.70833333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46289.44791666666</v>
+        <v>46289.70833333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46289.44791666666</v>
+        <v>46289.70833333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 10:13:10
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46288.16666666666</v>
+        <v>46288.41666666666</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46288.16666666666</v>
+        <v>46288.41666666666</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46288.16666666666</v>
+        <v>46288.41666666666</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-18 13:44:58
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4629,7 +4629,7 @@
         <v>4080</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>46283.27083333334</v>
+        <v>46283.22916666666</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
@@ -4676,7 +4676,7 @@
         <v>4080</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>46283.27083333334</v>
+        <v>46283.22916666666</v>
       </c>
       <c r="E30" t="n">
         <v>2</v>
@@ -4723,7 +4723,7 @@
         <v>4080</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>46283.27083333334</v>
+        <v>46283.22916666666</v>
       </c>
       <c r="E31" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-21 08:26:15
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46288.41666666666</v>
+        <v>46287.625</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46288.41666666666</v>
+        <v>46287.625</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46288.41666666666</v>
+        <v>46287.625</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-21 08:26:22
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46287.625</v>
+        <v>46288.13541666666</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46287.625</v>
+        <v>46288.13541666666</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46287.625</v>
+        <v>46288.13541666666</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-21 08:26:23
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46289.70833333334</v>
+        <v>46289.42708333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46289.70833333334</v>
+        <v>46289.42708333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46289.70833333334</v>
+        <v>46289.42708333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-21 12:09:32
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4756,130 +4756,16 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>363c5463-4dda-4b36-a1a0-607308debf39</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>TEST eliminare</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>180</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>46286.125</v>
-      </c>
-      <c r="E32" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H32" t="n">
-        <v>10</v>
-      </c>
-      <c r="J32" s="8" t="n">
-        <v>46283.40574331018</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>SUBITO</t>
-        </is>
-      </c>
+      <c r="D32" s="8" t="n"/>
+      <c r="J32" s="8" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>363c5463-4dda-4b36-a1a0-607308debf39</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>TEST eliminare</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>180</v>
-      </c>
-      <c r="D33" s="8" t="n">
-        <v>46286.125</v>
-      </c>
-      <c r="E33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Supporto</t>
-        </is>
-      </c>
-      <c r="H33" t="n">
-        <v>10</v>
-      </c>
-      <c r="J33" s="8" t="n">
-        <v>46283.40574331018</v>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>SUBITO</t>
-        </is>
-      </c>
+      <c r="D33" s="8" t="n"/>
+      <c r="J33" s="8" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>363c5463-4dda-4b36-a1a0-607308debf39</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>TEST eliminare</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>180</v>
-      </c>
-      <c r="D34" s="8" t="n">
-        <v>46286.125</v>
-      </c>
-      <c r="E34" t="n">
-        <v>3</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>B003</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H34" t="n">
-        <v>10</v>
-      </c>
-      <c r="J34" s="8" t="n">
-        <v>46283.40574331018</v>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>SUBITO</t>
-        </is>
-      </c>
+      <c r="D34" s="8" t="n"/>
+      <c r="J34" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-21 12:09:41
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46286.28125</v>
+        <v>46286.08333333334</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46286.28125</v>
+        <v>46286.08333333334</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46286.28125</v>
+        <v>46286.08333333334</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-21 12:09:44
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46286.08333333334</v>
+        <v>46286.41666666666</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46286.08333333334</v>
+        <v>46286.41666666666</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46286.08333333334</v>
+        <v>46286.41666666666</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-21 12:09:51
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46286.41666666666</v>
+        <v>46286.45833333334</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46286.41666666666</v>
+        <v>46286.45833333334</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46286.41666666666</v>
+        <v>46286.45833333334</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-21 12:09:53
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46286.45833333334</v>
+        <v>46286.47916666666</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46286.45833333334</v>
+        <v>46286.47916666666</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46286.45833333334</v>
+        <v>46286.47916666666</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-22 07:53:43
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -467,7 +467,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Caricata</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Caricata</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>B001</t>
+          <t>B006</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:04:42
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46289.42708333334</v>
+        <v>46291.40625</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46289.42708333334</v>
+        <v>46291.40625</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46289.42708333334</v>
+        <v>46291.40625</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:04:43
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46288.13541666666</v>
+        <v>46290.15625</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46288.13541666666</v>
+        <v>46290.15625</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46288.13541666666</v>
+        <v>46290.15625</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:04:50
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46286.47916666666</v>
+        <v>46288.82291666666</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46286.47916666666</v>
+        <v>46288.82291666666</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46286.47916666666</v>
+        <v>46288.82291666666</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:10:11
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -467,7 +467,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Caricata</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Caricata</t>
+          <t>Disponibile</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>B006</t>
+          <t>B001</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:12:47
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4065,7 +4065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4767,6 +4767,86 @@
       <c r="D34" s="8" t="n"/>
       <c r="J34" s="8" t="n"/>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>69052155-c1a0-43b9-8439-a6123a3ad699</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Phantom3</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>4082</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>770</v>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" s="8" t="n">
+        <v>46288.55052651343</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>69052155-c1a0-43b9-8439-a6123a3ad699</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Phantom3</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>4082</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>10</v>
+      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" s="8" t="n">
+        <v>46288.55052651343</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:19:14
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4065,7 +4065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4797,9 +4797,8 @@
       <c r="H35" t="n">
         <v>770</v>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" s="8" t="n">
-        <v>46288.55052651343</v>
+        <v>46288.55052651621</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -4837,11 +4836,90 @@
       <c r="H36" t="n">
         <v>10</v>
       </c>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" s="8" t="n">
-        <v>46288.55052651343</v>
+        <v>46288.55052651621</v>
       </c>
       <c r="K36" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>6f27b987-4a29-4e1c-b722-03e190820314</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Tappo+Mold1-francesca</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>480</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>23</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" s="8" t="n">
+        <v>46288.5550235603</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>6f27b987-4a29-4e1c-b722-03e190820314</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Tappo+Mold1-francesca</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>480</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>18</v>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" s="8" t="n">
+        <v>46288.5550235603</v>
+      </c>
+      <c r="K38" t="inlineStr">
         <is>
           <t>Quando possibile</t>
         </is>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:19:33
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4476,7 +4476,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46291.40625</v>
+        <v>46292.4375</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4523,7 +4523,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46291.40625</v>
+        <v>46292.4375</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4570,7 +4570,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46291.40625</v>
+        <v>46292.4375</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>
@@ -4875,9 +4875,8 @@
       <c r="H37" t="n">
         <v>23</v>
       </c>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" s="8" t="n">
-        <v>46288.5550235603</v>
+        <v>46288.55502356481</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -4915,9 +4914,8 @@
       <c r="H38" t="n">
         <v>18</v>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" s="8" t="n">
-        <v>46288.5550235603</v>
+        <v>46288.55502356481</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:19:34
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4281,7 +4281,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46290.15625</v>
+        <v>46291.14583333334</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4328,7 +4328,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46290.15625</v>
+        <v>46291.14583333334</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46290.15625</v>
+        <v>46291.14583333334</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:19:36
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46288.82291666666</v>
+        <v>46288.80208333334</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46288.82291666666</v>
+        <v>46288.80208333334</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46288.82291666666</v>
+        <v>46288.80208333334</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:19:38
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46288.80208333334</v>
+        <v>46289.80208333334</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46288.80208333334</v>
+        <v>46289.80208333334</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46288.80208333334</v>
+        <v>46289.80208333334</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:22:15
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4065,7 +4065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4923,6 +4923,86 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>90acf047-232c-4e50-9b5c-f9c02ee4f75f</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Supporti inferiori phantom</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>480</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>50</v>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" s="8" t="n">
+        <v>46288.55711080218</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>90acf047-232c-4e50-9b5c-f9c02ee4f75f</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Supporti inferiori phantom</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>480</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>9</v>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" s="8" t="n">
+        <v>46288.55711080218</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:22:31
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4140,7 +4140,7 @@
         <v>1860</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46289.80208333334</v>
+        <v>46286.09375</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -4187,7 +4187,7 @@
         <v>1860</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46289.80208333334</v>
+        <v>46286.09375</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -4234,7 +4234,7 @@
         <v>1860</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46289.80208333334</v>
+        <v>46286.09375</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -4953,9 +4953,8 @@
       <c r="H39" t="n">
         <v>50</v>
       </c>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" s="8" t="n">
-        <v>46288.55711080218</v>
+        <v>46288.55711079861</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -4993,9 +4992,8 @@
       <c r="H40" t="n">
         <v>9</v>
       </c>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" s="8" t="n">
-        <v>46288.55711080218</v>
+        <v>46288.55711079861</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:22:49
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -455,7 +455,7 @@
         <v>5000</v>
       </c>
       <c r="F2" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="G2">
         <f>MAX(0,E2-F2)</f>
@@ -501,7 +501,7 @@
         <v>1000</v>
       </c>
       <c r="F3" t="n">
-        <v>400</v>
+        <v>410</v>
       </c>
       <c r="G3">
         <f>MAX(0,E3-F3)</f>
@@ -547,7 +547,7 @@
         <v>1000</v>
       </c>
       <c r="F4" t="n">
-        <v>672</v>
+        <v>682</v>
       </c>
       <c r="G4">
         <f>MAX(0,E4-F4)</f>
@@ -3411,7 +3411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3886,6 +3886,132 @@
       </c>
       <c r="J14" s="8" t="n">
         <v>46282.72916666666</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n">
+        <v>46288.55694444444</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Phantom_part3</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1 parte superiore phantom</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>6279a9a1-9ecb-40fa-ae2e-13082f8b2c8d</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>4080</v>
+      </c>
+      <c r="J15" s="8" t="n">
+        <v>46283.22916666666</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>46288.55694444444</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Phantom_part3</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1 parte superiore phantom</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>6279a9a1-9ecb-40fa-ae2e-13082f8b2c8d</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>4080</v>
+      </c>
+      <c r="J16" s="8" t="n">
+        <v>46283.22916666666</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>46288.55694444444</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Phantom_part3</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>10</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1 parte superiore phantom</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>6279a9a1-9ecb-40fa-ae2e-13082f8b2c8d</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>4080</v>
+      </c>
+      <c r="J17" s="8" t="n">
+        <v>46283.22916666666</v>
       </c>
     </row>
   </sheetData>
@@ -4615,145 +4741,16 @@
       <c r="J28" s="8" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>547a8bc6-095c-45b5-b678-e3f9bc5105a0</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Phantom_part3</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>4080</v>
-      </c>
-      <c r="D29" s="8" t="n">
-        <v>46283.22916666666</v>
-      </c>
-      <c r="E29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H29" t="n">
-        <v>10</v>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>1 parte superiore phantom</t>
-        </is>
-      </c>
-      <c r="J29" s="8" t="n">
-        <v>46282.51013813657</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Quando possibile</t>
-        </is>
-      </c>
+      <c r="D29" s="8" t="n"/>
+      <c r="J29" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>547a8bc6-095c-45b5-b678-e3f9bc5105a0</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Phantom_part3</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>4080</v>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>46283.22916666666</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Supporto</t>
-        </is>
-      </c>
-      <c r="H30" t="n">
-        <v>10</v>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>1 parte superiore phantom</t>
-        </is>
-      </c>
-      <c r="J30" s="8" t="n">
-        <v>46282.51013813657</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Quando possibile</t>
-        </is>
-      </c>
+      <c r="D30" s="8" t="n"/>
+      <c r="J30" s="8" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>547a8bc6-095c-45b5-b678-e3f9bc5105a0</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Phantom_part3</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>4080</v>
-      </c>
-      <c r="D31" s="8" t="n">
-        <v>46283.22916666666</v>
-      </c>
-      <c r="E31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>B003</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H31" t="n">
-        <v>10</v>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>1 parte superiore phantom</t>
-        </is>
-      </c>
-      <c r="J31" s="8" t="n">
-        <v>46282.51013813657</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Quando possibile</t>
-        </is>
-      </c>
+      <c r="D31" s="8" t="n"/>
+      <c r="J31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="D32" s="8" t="n"/>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:22:55
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -455,7 +455,7 @@
         <v>5000</v>
       </c>
       <c r="F2" t="n">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="G2">
         <f>MAX(0,E2-F2)</f>
@@ -501,7 +501,7 @@
         <v>1000</v>
       </c>
       <c r="F3" t="n">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="G3">
         <f>MAX(0,E3-F3)</f>
@@ -547,7 +547,7 @@
         <v>1000</v>
       </c>
       <c r="F4" t="n">
-        <v>682</v>
+        <v>692</v>
       </c>
       <c r="G4">
         <f>MAX(0,E4-F4)</f>
@@ -3411,7 +3411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4012,6 +4012,132 @@
       </c>
       <c r="J17" s="8" t="n">
         <v>46283.22916666666</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>46288.55694444444</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ScatoleP1P5_inserti</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Scatole palpable da P1 a P5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>774fcc2e-eaac-4db2-bbfb-14259f5b254c</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>1860</v>
+      </c>
+      <c r="J18" s="8" t="n">
+        <v>46286.09375</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n">
+        <v>46288.55694444444</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ScatoleP1P5_inserti</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>10</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Scatole palpable da P1 a P5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>774fcc2e-eaac-4db2-bbfb-14259f5b254c</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>1860</v>
+      </c>
+      <c r="J19" s="8" t="n">
+        <v>46286.09375</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>46288.55694444444</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ScatoleP1P5_inserti</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>10</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Scatole palpable da P1 a P5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>774fcc2e-eaac-4db2-bbfb-14259f5b254c</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>1860</v>
+      </c>
+      <c r="J20" s="8" t="n">
+        <v>46286.09375</v>
       </c>
     </row>
   </sheetData>
@@ -4252,145 +4378,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>71d31883-77ba-4398-9dc9-8b313ee67220</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ScatoleP1P5_inserti</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1860</v>
-      </c>
-      <c r="D2" s="8" t="n">
-        <v>46286.09375</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>10</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Scatole palpable da P1 a P5</t>
-        </is>
-      </c>
-      <c r="J2" s="8" t="n">
-        <v>46282.43228212963</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>SUBITO</t>
-        </is>
-      </c>
+      <c r="D2" s="8" t="n"/>
+      <c r="J2" s="8" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>71d31883-77ba-4398-9dc9-8b313ee67220</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ScatoleP1P5_inserti</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1860</v>
-      </c>
-      <c r="D3" s="8" t="n">
-        <v>46286.09375</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Supporto</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>10</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Scatole palpable da P1 a P5</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="n">
-        <v>46282.43228212963</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>SUBITO</t>
-        </is>
-      </c>
+      <c r="D3" s="8" t="n"/>
+      <c r="J3" s="8" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>71d31883-77ba-4398-9dc9-8b313ee67220</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ScatoleP1P5_inserti</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1860</v>
-      </c>
-      <c r="D4" s="8" t="n">
-        <v>46286.09375</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>B003</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>10</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Scatole palpable da P1 a P5</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="n">
-        <v>46282.43228212963</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>SUBITO</t>
-        </is>
-      </c>
+      <c r="D4" s="8" t="n"/>
+      <c r="J4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:24:08
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4317,7 +4317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4995,6 +4995,86 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>33554ca2-afa2-4c26-b59a-ccf371ed3a61</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Colon Keychain</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>60</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>10</v>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" s="8" t="n">
+        <v>46288.55842799866</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>33554ca2-afa2-4c26-b59a-ccf371ed3a61</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Colon Keychain</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>60</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>10</v>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" s="8" t="n">
+        <v>46288.55842799866</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Quando possibile</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:25:16
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -5007,7 +5007,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>60</v>
+        <v>1620</v>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>46288.5625</v>
       </c>
       <c r="E41" t="n">
         <v>1</v>
@@ -5025,9 +5028,8 @@
       <c r="H41" t="n">
         <v>10</v>
       </c>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" s="8" t="n">
-        <v>46288.55842799866</v>
+        <v>46288.55842799768</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -5047,7 +5049,10 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>60</v>
+        <v>1620</v>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>46288.5625</v>
       </c>
       <c r="E42" t="n">
         <v>2</v>
@@ -5065,9 +5070,8 @@
       <c r="H42" t="n">
         <v>10</v>
       </c>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" s="8" t="n">
-        <v>46288.55842799866</v>
+        <v>46288.55842799768</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:25:24
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -5010,7 +5010,7 @@
         <v>1620</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>46288.5625</v>
+        <v>46288.6875</v>
       </c>
       <c r="E41" t="n">
         <v>1</v>
@@ -5052,7 +5052,7 @@
         <v>1620</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>46288.5625</v>
+        <v>46288.6875</v>
       </c>
       <c r="E42" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:25:29
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -5010,7 +5010,7 @@
         <v>1620</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>46288.6875</v>
+        <v>46288.70833333334</v>
       </c>
       <c r="E41" t="n">
         <v>1</v>
@@ -5052,7 +5052,7 @@
         <v>1620</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>46288.6875</v>
+        <v>46288.70833333334</v>
       </c>
       <c r="E42" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:26:10
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4404,7 +4404,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46291.14583333334</v>
+        <v>46290.22916666666</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4451,7 +4451,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46291.14583333334</v>
+        <v>46290.22916666666</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4498,7 +4498,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46291.14583333334</v>
+        <v>46290.22916666666</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:26:48
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4931,6 +4931,9 @@
       <c r="C39" t="n">
         <v>480</v>
       </c>
+      <c r="D39" s="8" t="n">
+        <v>46289.85416666666</v>
+      </c>
       <c r="E39" t="n">
         <v>1</v>
       </c>
@@ -4969,6 +4972,9 @@
       </c>
       <c r="C40" t="n">
         <v>480</v>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>46289.85416666666</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:26:59
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4932,7 +4932,7 @@
         <v>480</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>46289.85416666666</v>
+        <v>46291.53125</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -4974,7 +4974,7 @@
         <v>480</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>46289.85416666666</v>
+        <v>46291.53125</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:27:16
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4932,7 +4932,7 @@
         <v>480</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>46291.53125</v>
+        <v>46291.59375</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -4974,7 +4974,7 @@
         <v>480</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>46291.53125</v>
+        <v>46291.59375</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:27:27
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4853,6 +4853,9 @@
       <c r="C37" t="n">
         <v>480</v>
       </c>
+      <c r="D37" s="8" t="n">
+        <v>46292.04166666666</v>
+      </c>
       <c r="E37" t="n">
         <v>1</v>
       </c>
@@ -4891,6 +4894,9 @@
       </c>
       <c r="C38" t="n">
         <v>480</v>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>46292.04166666666</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:27:35
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4775,6 +4775,9 @@
       <c r="C35" t="n">
         <v>4082</v>
       </c>
+      <c r="D35" s="8" t="n">
+        <v>46293.76041666666</v>
+      </c>
       <c r="E35" t="n">
         <v>1</v>
       </c>
@@ -4813,6 +4816,9 @@
       </c>
       <c r="C36" t="n">
         <v>4082</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>46293.76041666666</v>
       </c>
       <c r="E36" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:37:24
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -5025,7 +5025,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1620</v>
+        <v>1920</v>
       </c>
       <c r="D41" s="8" t="n">
         <v>46288.70833333334</v>
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1620</v>
+        <v>1920</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>46288.70833333334</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:38:37
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -5025,7 +5025,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1920</v>
+        <v>2100</v>
       </c>
       <c r="D41" s="8" t="n">
         <v>46288.70833333334</v>
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1920</v>
+        <v>2100</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>46288.70833333334</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:38:46
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4944,7 +4944,7 @@
         <v>480</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>46291.59375</v>
+        <v>46291.67708333334</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -4986,7 +4986,7 @@
         <v>480</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>46291.59375</v>
+        <v>46291.67708333334</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:38:56
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4404,7 +4404,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46290.22916666666</v>
+        <v>46290.375</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4451,7 +4451,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46290.22916666666</v>
+        <v>46290.375</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4498,7 +4498,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46290.22916666666</v>
+        <v>46290.375</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:38:59
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4404,7 +4404,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46290.375</v>
+        <v>46290.33333333334</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4451,7 +4451,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46290.375</v>
+        <v>46290.33333333334</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4498,7 +4498,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46290.375</v>
+        <v>46290.33333333334</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:42:07
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -5025,7 +5025,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2100</v>
+        <v>2160</v>
       </c>
       <c r="D41" s="8" t="n">
         <v>46288.70833333334</v>
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2100</v>
+        <v>2160</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>46288.70833333334</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:45:17
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4404,7 +4404,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46290.33333333334</v>
+        <v>46290.34375</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4451,7 +4451,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46290.33333333334</v>
+        <v>46290.34375</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4498,7 +4498,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46290.33333333334</v>
+        <v>46290.34375</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:47:55
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4404,7 +4404,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46290.34375</v>
+        <v>46290.23958333334</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4451,7 +4451,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46290.34375</v>
+        <v>46290.23958333334</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4498,7 +4498,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46290.34375</v>
+        <v>46290.23958333334</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:48:04
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4775,9 +4775,7 @@
       <c r="C35" t="n">
         <v>4082</v>
       </c>
-      <c r="D35" s="8" t="n">
-        <v>46293.76041666666</v>
-      </c>
+      <c r="D35" s="8" t="n"/>
       <c r="E35" t="n">
         <v>1</v>
       </c>
@@ -4817,9 +4815,7 @@
       <c r="C36" t="n">
         <v>4082</v>
       </c>
-      <c r="D36" s="8" t="n">
-        <v>46293.76041666666</v>
-      </c>
+      <c r="D36" s="8" t="n"/>
       <c r="E36" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:48:09
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4598,9 +4598,7 @@
       <c r="C23" t="n">
         <v>1800</v>
       </c>
-      <c r="D23" s="8" t="n">
-        <v>46292.4375</v>
-      </c>
+      <c r="D23" s="8" t="n"/>
       <c r="E23" t="n">
         <v>1</v>
       </c>
@@ -4645,9 +4643,7 @@
       <c r="C24" t="n">
         <v>1800</v>
       </c>
-      <c r="D24" s="8" t="n">
-        <v>46292.4375</v>
-      </c>
+      <c r="D24" s="8" t="n"/>
       <c r="E24" t="n">
         <v>2</v>
       </c>
@@ -4692,9 +4688,7 @@
       <c r="C25" t="n">
         <v>1800</v>
       </c>
-      <c r="D25" s="8" t="n">
-        <v>46292.4375</v>
-      </c>
+      <c r="D25" s="8" t="n"/>
       <c r="E25" t="n">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:48:15
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4403,9 +4403,7 @@
       <c r="C5" t="n">
         <v>1800</v>
       </c>
-      <c r="D5" s="8" t="n">
-        <v>46290.23958333334</v>
-      </c>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" t="n">
         <v>1</v>
       </c>
@@ -4450,9 +4448,7 @@
       <c r="C6" t="n">
         <v>1800</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>46290.23958333334</v>
-      </c>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" t="n">
         <v>2</v>
       </c>
@@ -4497,9 +4493,7 @@
       <c r="C7" t="n">
         <v>1800</v>
       </c>
-      <c r="D7" s="8" t="n">
-        <v>46290.23958333334</v>
-      </c>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" t="n">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:48:26
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4927,9 +4927,7 @@
       <c r="C39" t="n">
         <v>480</v>
       </c>
-      <c r="D39" s="8" t="n">
-        <v>46291.67708333334</v>
-      </c>
+      <c r="D39" s="8" t="n"/>
       <c r="E39" t="n">
         <v>1</v>
       </c>
@@ -4969,9 +4967,7 @@
       <c r="C40" t="n">
         <v>480</v>
       </c>
-      <c r="D40" s="8" t="n">
-        <v>46291.67708333334</v>
-      </c>
+      <c r="D40" s="8" t="n"/>
       <c r="E40" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:48:29
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4843,9 +4843,7 @@
       <c r="C37" t="n">
         <v>480</v>
       </c>
-      <c r="D37" s="8" t="n">
-        <v>46292.04166666666</v>
-      </c>
+      <c r="D37" s="8" t="n"/>
       <c r="E37" t="n">
         <v>1</v>
       </c>
@@ -4885,9 +4883,7 @@
       <c r="C38" t="n">
         <v>480</v>
       </c>
-      <c r="D38" s="8" t="n">
-        <v>46292.04166666666</v>
-      </c>
+      <c r="D38" s="8" t="n"/>
       <c r="E38" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:48:56
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4763,7 +4763,9 @@
       <c r="C35" t="n">
         <v>4082</v>
       </c>
-      <c r="D35" s="8" t="n"/>
+      <c r="D35" s="8" t="n">
+        <v>46290.34375</v>
+      </c>
       <c r="E35" t="n">
         <v>1</v>
       </c>
@@ -4803,7 +4805,9 @@
       <c r="C36" t="n">
         <v>4082</v>
       </c>
-      <c r="D36" s="8" t="n"/>
+      <c r="D36" s="8" t="n">
+        <v>46290.34375</v>
+      </c>
       <c r="E36" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:49:11
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4847,7 +4847,9 @@
       <c r="C37" t="n">
         <v>480</v>
       </c>
-      <c r="D37" s="8" t="n"/>
+      <c r="D37" s="8" t="n">
+        <v>46293.21875</v>
+      </c>
       <c r="E37" t="n">
         <v>1</v>
       </c>
@@ -4887,7 +4889,9 @@
       <c r="C38" t="n">
         <v>480</v>
       </c>
-      <c r="D38" s="8" t="n"/>
+      <c r="D38" s="8" t="n">
+        <v>46293.21875</v>
+      </c>
       <c r="E38" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:49:20
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4848,7 +4848,7 @@
         <v>480</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>46293.21875</v>
+        <v>46293.35416666666</v>
       </c>
       <c r="E37" t="n">
         <v>1</v>
@@ -4890,7 +4890,7 @@
         <v>480</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>46293.21875</v>
+        <v>46293.35416666666</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:49:26
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4931,7 +4931,9 @@
       <c r="C39" t="n">
         <v>480</v>
       </c>
-      <c r="D39" s="8" t="n"/>
+      <c r="D39" s="8" t="n">
+        <v>46293.70833333334</v>
+      </c>
       <c r="E39" t="n">
         <v>1</v>
       </c>
@@ -4971,7 +4973,9 @@
       <c r="C40" t="n">
         <v>480</v>
       </c>
-      <c r="D40" s="8" t="n"/>
+      <c r="D40" s="8" t="n">
+        <v>46293.70833333334</v>
+      </c>
       <c r="E40" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:49:32
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4592,7 +4592,9 @@
       <c r="C23" t="n">
         <v>1800</v>
       </c>
-      <c r="D23" s="8" t="n"/>
+      <c r="D23" s="8" t="n">
+        <v>46294.34375</v>
+      </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
@@ -4637,7 +4639,9 @@
       <c r="C24" t="n">
         <v>1800</v>
       </c>
-      <c r="D24" s="8" t="n"/>
+      <c r="D24" s="8" t="n">
+        <v>46294.34375</v>
+      </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
@@ -4682,7 +4686,9 @@
       <c r="C25" t="n">
         <v>1800</v>
       </c>
-      <c r="D25" s="8" t="n"/>
+      <c r="D25" s="8" t="n">
+        <v>46294.34375</v>
+      </c>
       <c r="E25" t="n">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:49:38
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4938,7 +4938,7 @@
         <v>480</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>46293.70833333334</v>
+        <v>46295.63541666666</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -4980,7 +4980,7 @@
         <v>480</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>46293.70833333334</v>
+        <v>46295.63541666666</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:49:46
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4593,7 +4593,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46294.34375</v>
+        <v>46296.13541666666</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4640,7 +4640,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46294.34375</v>
+        <v>46296.13541666666</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4687,7 +4687,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46294.34375</v>
+        <v>46296.13541666666</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:49:50
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4938,7 +4938,7 @@
         <v>480</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>46295.63541666666</v>
+        <v>46293.72916666666</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -4980,7 +4980,7 @@
         <v>480</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>46295.63541666666</v>
+        <v>46293.72916666666</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:49:55
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4593,7 +4593,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46296.13541666666</v>
+        <v>46294.33333333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4640,7 +4640,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46296.13541666666</v>
+        <v>46294.33333333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4687,7 +4687,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46296.13541666666</v>
+        <v>46294.33333333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:50:01
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4403,7 +4403,9 @@
       <c r="C5" t="n">
         <v>1800</v>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="8" t="n">
+        <v>46295.625</v>
+      </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
@@ -4448,7 +4450,9 @@
       <c r="C6" t="n">
         <v>1800</v>
       </c>
-      <c r="D6" s="8" t="n"/>
+      <c r="D6" s="8" t="n">
+        <v>46295.625</v>
+      </c>
       <c r="E6" t="n">
         <v>2</v>
       </c>
@@ -4493,7 +4497,9 @@
       <c r="C7" t="n">
         <v>1800</v>
       </c>
-      <c r="D7" s="8" t="n"/>
+      <c r="D7" s="8" t="n">
+        <v>46295.625</v>
+      </c>
       <c r="E7" t="n">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-23 13:50:08
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4404,7 +4404,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46295.625</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4451,7 +4451,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46295.625</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4498,7 +4498,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46295.625</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-25 08:44:37
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4404,7 +4404,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46295.66666666666</v>
+        <v>46296.63541666666</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4451,7 +4451,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46295.66666666666</v>
+        <v>46296.63541666666</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4498,7 +4498,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46295.66666666666</v>
+        <v>46296.63541666666</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-25 08:44:39
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4404,7 +4404,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46296.63541666666</v>
+        <v>46295.64583333334</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4451,7 +4451,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46296.63541666666</v>
+        <v>46295.64583333334</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4498,7 +4498,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46296.63541666666</v>
+        <v>46295.64583333334</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 09:35:51
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4404,7 +4404,7 @@
         <v>1800</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46295.64583333334</v>
+        <v>46296.71875</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -4451,7 +4451,7 @@
         <v>1800</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46295.64583333334</v>
+        <v>46296.71875</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -4498,7 +4498,7 @@
         <v>1800</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46295.64583333334</v>
+        <v>46296.71875</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 09:35:57
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4599,7 +4599,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46294.33333333334</v>
+        <v>46295.4375</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4646,7 +4646,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46294.33333333334</v>
+        <v>46295.4375</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4693,7 +4693,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46294.33333333334</v>
+        <v>46295.4375</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 09:36:04
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4599,7 +4599,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46295.4375</v>
+        <v>46295.36458333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4646,7 +4646,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46295.4375</v>
+        <v>46295.36458333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4693,7 +4693,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46295.4375</v>
+        <v>46295.36458333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 09:36:13
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4944,7 +4944,7 @@
         <v>480</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>46293.72916666666</v>
+        <v>46294.375</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -4986,7 +4986,7 @@
         <v>480</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>46293.72916666666</v>
+        <v>46294.375</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 12:14:13
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4860,7 +4860,7 @@
         <v>480</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>46293.35416666666</v>
+        <v>46295</v>
       </c>
       <c r="E37" t="n">
         <v>1</v>
@@ -4902,7 +4902,7 @@
         <v>480</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>46293.35416666666</v>
+        <v>46295</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 12:14:21
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4599,7 +4599,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46295.36458333334</v>
+        <v>46295.39583333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4646,7 +4646,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46295.36458333334</v>
+        <v>46295.39583333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4693,7 +4693,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46295.36458333334</v>
+        <v>46295.39583333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 12:14:49
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4944,7 +4944,7 @@
         <v>480</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>46294.375</v>
+        <v>46294.30208333334</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -4986,7 +4986,7 @@
         <v>480</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>46294.375</v>
+        <v>46294.30208333334</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 12:14:56
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4944,7 +4944,7 @@
         <v>480</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>46294.30208333334</v>
+        <v>46294.29166666666</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -4986,7 +4986,7 @@
         <v>480</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>46294.30208333334</v>
+        <v>46294.29166666666</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 12:14:59
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4860,7 +4860,7 @@
         <v>480</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="E37" t="n">
         <v>1</v>
@@ -4902,7 +4902,7 @@
         <v>480</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 12:15:04
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -4599,7 +4599,7 @@
         <v>1800</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46295.39583333334</v>
+        <v>46294.64583333334</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4646,7 +4646,7 @@
         <v>1800</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46295.39583333334</v>
+        <v>46294.64583333334</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4693,7 +4693,7 @@
         <v>1800</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46295.39583333334</v>
+        <v>46294.64583333334</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 12:15:19
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -455,7 +455,7 @@
         <v>5000</v>
       </c>
       <c r="F2" t="n">
-        <v>92</v>
+        <v>862</v>
       </c>
       <c r="G2">
         <f>MAX(0,E2-F2)</f>
@@ -501,7 +501,7 @@
         <v>1000</v>
       </c>
       <c r="F3" t="n">
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="G3">
         <f>MAX(0,E3-F3)</f>
@@ -3411,7 +3411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4138,6 +4138,82 @@
       </c>
       <c r="J20" s="8" t="n">
         <v>46286.09375</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
+        <v>46294.51041666666</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Phantom3</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>770</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>60988efd-fbd2-4d1a-821b-10b4cbdb5c09</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>4082</v>
+      </c>
+      <c r="J21" s="8" t="n">
+        <v>46290.34375</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>46294.51041666666</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Phantom3</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>60988efd-fbd2-4d1a-821b-10b4cbdb5c09</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>4082</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>46290.34375</v>
       </c>
     </row>
   </sheetData>
@@ -4762,88 +4838,12 @@
       <c r="J34" s="8" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>69052155-c1a0-43b9-8439-a6123a3ad699</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Phantom3</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>4082</v>
-      </c>
-      <c r="D35" s="8" t="n">
-        <v>46290.34375</v>
-      </c>
-      <c r="E35" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H35" t="n">
-        <v>770</v>
-      </c>
-      <c r="J35" s="8" t="n">
-        <v>46288.55052651621</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Quando possibile</t>
-        </is>
-      </c>
+      <c r="D35" s="8" t="n"/>
+      <c r="J35" s="8" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>69052155-c1a0-43b9-8439-a6123a3ad699</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Phantom3</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>4082</v>
-      </c>
-      <c r="D36" s="8" t="n">
-        <v>46290.34375</v>
-      </c>
-      <c r="E36" t="n">
-        <v>2</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Supporto</t>
-        </is>
-      </c>
-      <c r="H36" t="n">
-        <v>10</v>
-      </c>
-      <c r="J36" s="8" t="n">
-        <v>46288.55052651621</v>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Quando possibile</t>
-        </is>
-      </c>
+      <c r="D36" s="8" t="n"/>
+      <c r="J36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">

</xml_diff>

<commit_message>
Aggiorna dati dashboard · 2026-09-29 12:15:29
</commit_message>
<xml_diff>
--- a/Tracker_Filament_Dashboard.xlsx
+++ b/Tracker_Filament_Dashboard.xlsx
@@ -455,7 +455,7 @@
         <v>5000</v>
       </c>
       <c r="F2" t="n">
-        <v>862</v>
+        <v>872</v>
       </c>
       <c r="G2">
         <f>MAX(0,E2-F2)</f>
@@ -501,7 +501,7 @@
         <v>1000</v>
       </c>
       <c r="F3" t="n">
-        <v>430</v>
+        <v>440</v>
       </c>
       <c r="G3">
         <f>MAX(0,E3-F3)</f>
@@ -3411,7 +3411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4165,7 +4165,6 @@
       <c r="F21" t="n">
         <v>770</v>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>60988efd-fbd2-4d1a-821b-10b4cbdb5c09</t>
@@ -4203,7 +4202,6 @@
       <c r="F22" t="n">
         <v>10</v>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>60988efd-fbd2-4d1a-821b-10b4cbdb5c09</t>
@@ -4214,6 +4212,82 @@
       </c>
       <c r="J22" s="8" t="n">
         <v>46290.34375</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
+        <v>46294.51041666666</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Colon Keychain</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ABS</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>10</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>17d9fa96-c4b9-482e-9e7e-bb1603cb0db1</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>2160</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>46288.70833333334</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n">
+        <v>46294.51041666666</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Colon Keychain</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Supporto</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>10</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>17d9fa96-c4b9-482e-9e7e-bb1603cb0db1</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>2160</v>
+      </c>
+      <c r="J24" s="8" t="n">
+        <v>46288.70833333334</v>
       </c>
     </row>
   </sheetData>
@@ -5014,88 +5088,12 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>33554ca2-afa2-4c26-b59a-ccf371ed3a61</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Colon Keychain</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>2160</v>
-      </c>
-      <c r="D41" s="8" t="n">
-        <v>46288.70833333334</v>
-      </c>
-      <c r="E41" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>ABS</t>
-        </is>
-      </c>
-      <c r="H41" t="n">
-        <v>10</v>
-      </c>
-      <c r="J41" s="8" t="n">
-        <v>46288.55842799768</v>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Quando possibile</t>
-        </is>
-      </c>
+      <c r="D41" s="8" t="n"/>
+      <c r="J41" s="8" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>33554ca2-afa2-4c26-b59a-ccf371ed3a61</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Colon Keychain</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>2160</v>
-      </c>
-      <c r="D42" s="8" t="n">
-        <v>46288.70833333334</v>
-      </c>
-      <c r="E42" t="n">
-        <v>2</v>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Supporto</t>
-        </is>
-      </c>
-      <c r="H42" t="n">
-        <v>10</v>
-      </c>
-      <c r="J42" s="8" t="n">
-        <v>46288.55842799768</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Quando possibile</t>
-        </is>
-      </c>
+      <c r="D42" s="8" t="n"/>
+      <c r="J42" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>